<commit_message>
Add total quantity sold to rport
</commit_message>
<xml_diff>
--- a/sales_report.xlsx
+++ b/sales_report.xlsx
@@ -17,13 +17,16 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -34,7 +37,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -42,12 +45,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -413,231 +425,51 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F9"/>
+  <dimension ref="A1:B4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Data </t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>Product</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>Category</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>Quantity</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>Price</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>Total</t>
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Sales</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Values</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="n">
-        <v>46031</v>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Laptop</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>Electronics</t>
-        </is>
-      </c>
-      <c r="D2" t="n">
-        <v>2</v>
-      </c>
-      <c r="E2" t="n">
-        <v>15000</v>
-      </c>
-      <c r="F2" t="n">
-        <v>30000</v>
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Total Quantity Sold</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>39</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="n">
-        <v>46062</v>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Mouse</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>Electronics</t>
-        </is>
-      </c>
-      <c r="D3" t="n">
-        <v>10</v>
-      </c>
-      <c r="E3" t="n">
-        <v>500</v>
-      </c>
-      <c r="F3" t="n">
-        <v>5000</v>
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Total Sales</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>119500</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="n">
-        <v>46090</v>
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Top Productt</t>
+        </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Chair</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>Furniture</t>
-        </is>
-      </c>
-      <c r="D4" t="n">
-        <v>5</v>
-      </c>
-      <c r="E4" t="n">
-        <v>2000</v>
-      </c>
-      <c r="F4" t="n">
-        <v>10000</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="n">
-        <v>46121</v>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Keyboard</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>Electronics</t>
-        </is>
-      </c>
-      <c r="D5" t="n">
-        <v>6</v>
-      </c>
-      <c r="E5" t="n">
-        <v>500</v>
-      </c>
-      <c r="F5" t="n">
-        <v>3000</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="n">
-        <v>46151</v>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>Desk</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>Furniture</t>
-        </is>
-      </c>
-      <c r="D6" t="n">
-        <v>3</v>
-      </c>
-      <c r="E6" t="n">
-        <v>9000</v>
-      </c>
-      <c r="F6" t="n">
-        <v>27000</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="n">
-        <v>46182</v>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
           <t>Monitor</t>
         </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>Electronics</t>
-        </is>
-      </c>
-      <c r="D7" t="n">
-        <v>4</v>
-      </c>
-      <c r="E7" t="n">
-        <v>8000</v>
-      </c>
-      <c r="F7" t="n">
-        <v>32000</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="n">
-        <v>46212</v>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>Chair</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>Furniture</t>
-        </is>
-      </c>
-      <c r="D8" t="n">
-        <v>4</v>
-      </c>
-      <c r="E8" t="n">
-        <v>2500</v>
-      </c>
-      <c r="F8" t="n">
-        <v>10000</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="n">
-        <v>46243</v>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>Mouse</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>Electronics</t>
-        </is>
-      </c>
-      <c r="D9" t="n">
-        <v>5</v>
-      </c>
-      <c r="E9" t="n">
-        <v>500</v>
-      </c>
-      <c r="F9" t="n">
-        <v>2500</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add Excel summary sheet
</commit_message>
<xml_diff>
--- a/sales_report.xlsx
+++ b/sales_report.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Summary" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,16 +17,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -37,7 +34,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -45,21 +42,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -425,16 +413,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B4"/>
+  <dimension ref="A1:B6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Sales</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Values</t>
         </is>
@@ -463,13 +451,33 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Top Productt</t>
+          <t>Top Product</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
           <t>Monitor</t>
         </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Electronics Sales</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>72500</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Furniture Sales</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>47000</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Upgrade Excel report with formatting and charts
</commit_message>
<xml_diff>
--- a/sales_report.xlsx
+++ b/sales_report.xlsx
@@ -8,6 +8,9 @@
   </bookViews>
   <sheets>
     <sheet name="Summary" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Category Sales" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Raw Data" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Product Sales" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,7 +20,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -25,16 +28,25 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001F4E78"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -42,12 +54,23 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -122,6 +145,284 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Sales by Category</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <barChart>
+        <barDir val="col"/>
+        <grouping val="clustered"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Category Sales'!B1</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Category Sales'!$A$2:$A$3</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Category Sales'!$B$2:$B$3</f>
+            </numRef>
+          </val>
+        </ser>
+        <gapWidth val="150"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </barChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Category</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Total Sales</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Sales by Product</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <barChart>
+        <barDir val="col"/>
+        <grouping val="clustered"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Product Sales'!B1</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Product Sales'!$A$2:$A$7</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Product Sales'!$B$2:$B$7</f>
+            </numRef>
+          </val>
+        </ser>
+        <gapWidth val="150"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </barChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Product</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Total Sales</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>3</col>
+      <colOff>0</colOff>
+      <row>1</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="5400000" cy="2700000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="1" name="Chart 1"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>3</col>
+      <colOff>0</colOff>
+      <row>1</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="5400000" cy="2700000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="1" name="Chart 1"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -413,74 +714,446 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B6"/>
+  <dimension ref="A1:B4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Sales</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Values</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Total Quantity Sold</t>
         </is>
       </c>
-      <c r="B2" t="n">
+      <c r="B2" s="3" t="n">
         <v>39</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="2" t="inlineStr">
         <is>
           <t>Total Sales</t>
         </is>
       </c>
-      <c r="B3" t="n">
+      <c r="B3" s="3" t="n">
         <v>119500</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" s="2" t="inlineStr">
         <is>
           <t>Top Product</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="B4" s="2" t="inlineStr">
         <is>
           <t>Monitor</t>
         </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Electronics Sales</t>
-        </is>
-      </c>
-      <c r="B5" t="n">
-        <v>72500</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Furniture Sales</t>
-        </is>
-      </c>
-      <c r="B6" t="n">
-        <v>47000</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Category</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Total Sales</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Electronics</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="n">
+        <v>72500</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Furniture</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="n">
+        <v>47000</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F9"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="15" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Data </t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Product</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Category</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Quantity</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Price</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="n">
+        <v>46031</v>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Laptop</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Electronics</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="E2" s="2" t="n">
+        <v>15000</v>
+      </c>
+      <c r="F2" s="2" t="n">
+        <v>30000</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="n">
+        <v>46062</v>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Mouse</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>Electronics</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="E3" s="2" t="n">
+        <v>500</v>
+      </c>
+      <c r="F3" s="2" t="n">
+        <v>5000</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="n">
+        <v>46090</v>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Chair</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Furniture</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="E4" s="2" t="n">
+        <v>2000</v>
+      </c>
+      <c r="F4" s="2" t="n">
+        <v>10000</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="n">
+        <v>46121</v>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Keyboard</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>Electronics</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="E5" s="2" t="n">
+        <v>500</v>
+      </c>
+      <c r="F5" s="2" t="n">
+        <v>3000</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="n">
+        <v>46151</v>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Desk</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>Furniture</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="E6" s="2" t="n">
+        <v>9000</v>
+      </c>
+      <c r="F6" s="2" t="n">
+        <v>27000</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="n">
+        <v>46182</v>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Monitor</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>Electronics</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="E7" s="2" t="n">
+        <v>8000</v>
+      </c>
+      <c r="F7" s="2" t="n">
+        <v>32000</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="n">
+        <v>46212</v>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Chair</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>Furniture</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="E8" s="2" t="n">
+        <v>2500</v>
+      </c>
+      <c r="F8" s="2" t="n">
+        <v>10000</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="n">
+        <v>46243</v>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>Mouse</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>Electronics</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="E9" s="2" t="n">
+        <v>500</v>
+      </c>
+      <c r="F9" s="2" t="n">
+        <v>2500</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Product</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Total Sales</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Monitor</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="n">
+        <v>32000</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Laptop</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="n">
+        <v>30000</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Desk</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="n">
+        <v>27000</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Chair</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="n">
+        <v>20000</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>Mouse</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="n">
+        <v>7500</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>Keyboard</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="n">
+        <v>3000</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Add GUI to Excel Report Generator
</commit_message>
<xml_diff>
--- a/sales_report.xlsx
+++ b/sales_report.xlsx
@@ -25,13 +25,16 @@
     <numFmt numFmtId="165" formatCode="YYYY-MM-DD HH:MM:SS"/>
     <numFmt numFmtId="166" formatCode="dd-mm-yyyy"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
     <font>
       <b val="1"/>
@@ -71,7 +74,7 @@
   </cellStyleXfs>
   <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>

</xml_diff>

<commit_message>
Simplify GUI input workflow
</commit_message>
<xml_diff>
--- a/sales_report.xlsx
+++ b/sales_report.xlsx
@@ -10,8 +10,8 @@
     <sheet name="Summary" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Category Sales" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Product Sales" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Raw Data" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Monthly Sales" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Monthly Sales" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Raw Data" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -23,7 +23,7 @@
   <numFmts count="3">
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
     <numFmt numFmtId="165" formatCode="YYYY-MM-DD HH:MM:SS"/>
-    <numFmt numFmtId="166" formatCode="dd-mm-yyyy"/>
+    <numFmt numFmtId="166" formatCode="dd-mmm-yyyy"/>
   </numFmts>
   <fonts count="3">
     <font>
@@ -72,7 +72,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -80,6 +80,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -583,11 +584,11 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="RawDataTable" displayName="RawDataTable" ref="A1:F9" headerRowCount="1">
   <autoFilter ref="A1:F9"/>
   <tableColumns count="6">
-    <tableColumn id="1" name="Date"/>
-    <tableColumn id="2" name="Product"/>
-    <tableColumn id="3" name="Category"/>
-    <tableColumn id="4" name="Quantity"/>
-    <tableColumn id="5" name="Price"/>
+    <tableColumn id="1" name="Product"/>
+    <tableColumn id="2" name="Category"/>
+    <tableColumn id="3" name="Quantity"/>
+    <tableColumn id="4" name="Price"/>
+    <tableColumn id="5" name="Date"/>
     <tableColumn id="6" name="Total"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -1096,6 +1097,117 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:B9"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Month</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>2026-01</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="n">
+        <v>30000</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>2026-02</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="n">
+        <v>5000</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>2026-03</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="n">
+        <v>10000</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>2026-04</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="n">
+        <v>3000</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>2026-05</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="n">
+        <v>27000</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>2026-06</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="n">
+        <v>32000</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="n">
+        <v>10000</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>2026-08</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="n">
+        <v>2500</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:F9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -1110,29 +1222,29 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
+          <t>Product</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Category</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Quantity</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Price</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
           <t>Date</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Product</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Category</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>Quantity</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>Price</t>
-        </is>
-      </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Total</t>
@@ -1140,192 +1252,192 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="4" t="n">
+      <c r="A2" s="4" t="inlineStr">
+        <is>
+          <t>Laptop</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Electronics</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="D2" s="2" t="n">
+        <v>15000</v>
+      </c>
+      <c r="E2" s="5" t="n">
         <v>46031</v>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>Laptop</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>Electronics</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="E2" s="2" t="n">
-        <v>15000</v>
       </c>
       <c r="F2" s="2" t="n">
         <v>30000</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="4" t="n">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>Mouse</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Electronics</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="D3" s="2" t="n">
+        <v>500</v>
+      </c>
+      <c r="E3" s="5" t="n">
         <v>46062</v>
-      </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>Mouse</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>Electronics</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="n">
-        <v>10</v>
-      </c>
-      <c r="E3" s="2" t="n">
-        <v>500</v>
       </c>
       <c r="F3" s="2" t="n">
         <v>5000</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="4" t="n">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Chair</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Furniture</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="D4" s="2" t="n">
+        <v>2000</v>
+      </c>
+      <c r="E4" s="5" t="n">
         <v>46090</v>
-      </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>Chair</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>Furniture</t>
-        </is>
-      </c>
-      <c r="D4" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="E4" s="2" t="n">
-        <v>2000</v>
       </c>
       <c r="F4" s="2" t="n">
         <v>10000</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="4" t="n">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Keyboard</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Electronics</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="D5" s="2" t="n">
+        <v>500</v>
+      </c>
+      <c r="E5" s="5" t="n">
         <v>46121</v>
-      </c>
-      <c r="B5" s="2" t="inlineStr">
-        <is>
-          <t>Keyboard</t>
-        </is>
-      </c>
-      <c r="C5" s="2" t="inlineStr">
-        <is>
-          <t>Electronics</t>
-        </is>
-      </c>
-      <c r="D5" s="2" t="n">
-        <v>6</v>
-      </c>
-      <c r="E5" s="2" t="n">
-        <v>500</v>
       </c>
       <c r="F5" s="2" t="n">
         <v>3000</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="4" t="n">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>Desk</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Furniture</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="D6" s="2" t="n">
+        <v>9000</v>
+      </c>
+      <c r="E6" s="5" t="n">
         <v>46151</v>
-      </c>
-      <c r="B6" s="2" t="inlineStr">
-        <is>
-          <t>Desk</t>
-        </is>
-      </c>
-      <c r="C6" s="2" t="inlineStr">
-        <is>
-          <t>Furniture</t>
-        </is>
-      </c>
-      <c r="D6" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="E6" s="2" t="n">
-        <v>9000</v>
       </c>
       <c r="F6" s="2" t="n">
         <v>27000</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="4" t="n">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>Monitor</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Electronics</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="D7" s="2" t="n">
+        <v>8000</v>
+      </c>
+      <c r="E7" s="5" t="n">
         <v>46182</v>
-      </c>
-      <c r="B7" s="2" t="inlineStr">
-        <is>
-          <t>Monitor</t>
-        </is>
-      </c>
-      <c r="C7" s="2" t="inlineStr">
-        <is>
-          <t>Electronics</t>
-        </is>
-      </c>
-      <c r="D7" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="E7" s="2" t="n">
-        <v>8000</v>
       </c>
       <c r="F7" s="2" t="n">
         <v>32000</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="4" t="n">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>Chair</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Furniture</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="D8" s="2" t="n">
+        <v>2500</v>
+      </c>
+      <c r="E8" s="5" t="n">
         <v>46212</v>
-      </c>
-      <c r="B8" s="2" t="inlineStr">
-        <is>
-          <t>Chair</t>
-        </is>
-      </c>
-      <c r="C8" s="2" t="inlineStr">
-        <is>
-          <t>Furniture</t>
-        </is>
-      </c>
-      <c r="D8" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="E8" s="2" t="n">
-        <v>2500</v>
       </c>
       <c r="F8" s="2" t="n">
         <v>10000</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="4" t="n">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>Mouse</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>Electronics</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="D9" s="2" t="n">
+        <v>500</v>
+      </c>
+      <c r="E9" s="5" t="n">
         <v>46243</v>
-      </c>
-      <c r="B9" s="2" t="inlineStr">
-        <is>
-          <t>Mouse</t>
-        </is>
-      </c>
-      <c r="C9" s="2" t="inlineStr">
-        <is>
-          <t>Electronics</t>
-        </is>
-      </c>
-      <c r="D9" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="E9" s="2" t="n">
-        <v>500</v>
       </c>
       <c r="F9" s="2" t="n">
         <v>2500</v>
@@ -1337,115 +1449,4 @@
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
   </tableParts>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:B9"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="20" customWidth="1" min="1" max="1"/>
-    <col width="20" customWidth="1" min="2" max="2"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Month</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Total</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>2026-01</t>
-        </is>
-      </c>
-      <c r="B2" s="3" t="n">
-        <v>30000</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>2026-02</t>
-        </is>
-      </c>
-      <c r="B3" s="3" t="n">
-        <v>5000</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>2026-03</t>
-        </is>
-      </c>
-      <c r="B4" s="3" t="n">
-        <v>10000</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>2026-04</t>
-        </is>
-      </c>
-      <c r="B5" s="3" t="n">
-        <v>3000</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>2026-05</t>
-        </is>
-      </c>
-      <c r="B6" s="3" t="n">
-        <v>27000</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="2" t="inlineStr">
-        <is>
-          <t>2026-06</t>
-        </is>
-      </c>
-      <c r="B7" s="3" t="n">
-        <v>32000</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="2" t="inlineStr">
-        <is>
-          <t>2026-07</t>
-        </is>
-      </c>
-      <c r="B8" s="3" t="n">
-        <v>10000</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="2" t="inlineStr">
-        <is>
-          <t>2026-08</t>
-        </is>
-      </c>
-      <c r="B9" s="3" t="n">
-        <v>2500</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
Finalize excel report generator
</commit_message>
<xml_diff>
--- a/sales_report.xlsx
+++ b/sales_report.xlsx
@@ -25,16 +25,13 @@
     <numFmt numFmtId="165" formatCode="YYYY-MM-DD HH:MM:SS"/>
     <numFmt numFmtId="166" formatCode="dd-mmm-yyyy"/>
   </numFmts>
-  <fonts count="3">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
     <font>
       <b val="1"/>
@@ -74,7 +71,7 @@
   </cellStyleXfs>
   <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>

</xml_diff>